<commit_message>
Figura 09: grosor promedio solo con --verbose (C4)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01NzBfV3TEaZuiM5M4wepfB7
</commit_message>
<xml_diff>
--- a/data/processed_data/Video_063_CTRL1_5V/contracciones_Video_063_CTRL1_5V.xlsx
+++ b/data/processed_data/Video_063_CTRL1_5V/contracciones_Video_063_CTRL1_5V.xlsx
@@ -24,16 +24,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -44,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -52,21 +49,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -436,22 +424,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>k</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>umbral_px</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>eventos</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>falsos_control</t>
         </is>
@@ -794,322 +782,322 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>canal</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>fps</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>n_frames</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>duracion_s</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>signo</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ruido_canal_px</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>ruido_grosor_px</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>n_eventos</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>k_usado</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>k_automatico</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>hay_meseta</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>meseta_motivo</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>meseta_k_rango</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>conteo_reportable</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>intervalo_mediano_s</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>amplitud_traslacion_px</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>ritmo</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>fps_medido</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>adelgazamiento_px</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>adelgazamiento_sigma</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>retardo_adelgazamiento_s</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>cociente_adelg_trasl_pct</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>adelgazamiento_robusto_px</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>adelgazamiento_robusto_sigma</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>cociente_robusto_pct</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>blur_px</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>blur_sigma</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>cinetica_grupo_principal</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>cinetica_min_frames</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>n_eventos_cinetica</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>amplitud_relativa_pct</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>amplitud_relativa_iqr_pct</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>ttp_n_eventos</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>ttp_n_medibles</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>ttp_frames_mediana</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>ttp_reportable</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>ttp_s</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>ttp_iqr_s</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>ttp_cota_inf_s</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>ttp_cota_sup_s</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>rt50_n_eventos</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>rt50_n_medibles</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>rt50_frames_mediana</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>rt50_reportable</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>rt50_s</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>rt50_iqr_s</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>rt50_cota_inf_s</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>rt50_cota_sup_s</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>cinetica_motivo</t>
         </is>
       </c>
-      <c r="AX1" s="1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>fotogramas_sin_medida</t>
         </is>
       </c>
-      <c r="AY1" s="1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>fotogramas_sin_medida_pct</t>
         </is>
       </c>
-      <c r="AZ1" s="1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>fotogramas_low_quality</t>
         </is>
       </c>
-      <c r="BA1" s="1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>eventos_junto_a_hueco</t>
         </is>
       </c>
-      <c r="BB1" s="1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>eventos_junto_al_borde</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>win_s_usado</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>win_s_automatico</t>
         </is>
       </c>
-      <c r="BE1" s="1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>duracion_evento_max_s</t>
         </is>
       </c>
-      <c r="BF1" s="1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>ventana_corta</t>
         </is>
       </c>
-      <c r="BG1" s="1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>conteo_por_ventana</t>
         </is>
       </c>
-      <c r="BH1" s="1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>conteo_estable_ventana</t>
         </is>
       </c>
-      <c r="BI1" s="1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>mesetas</t>
         </is>
       </c>
-      <c r="BJ1" s="1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>ruido_borde_sup_px</t>
         </is>
       </c>
-      <c r="BK1" s="1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>ruido_borde_inf_px</t>
         </is>
       </c>
-      <c r="BL1" s="1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>cociente_ruido_bordes</t>
         </is>
@@ -1351,52 +1339,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>grupo</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>n</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>t_inicio_s</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>t_fin_s</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>intervalo_mediano_s</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>intervalo_IQR_s</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>frecuencia_mediana_Hz</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>CV_intervalo_pct</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>amplitud_mediana_px</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>amplitud_IQR_px</t>
         </is>
@@ -1477,87 +1465,87 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>tren</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>busqueda</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>veredicto</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>clasificacion</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>periodo_s</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>periodo_err_s</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>frecuencia_Hz</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>jitter_ms</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>z</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>p_valor</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>n_eventos_tren</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>n_ranuras</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>captura_pct</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>n_dudosos</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>n_sacados_tiempo_amplitud</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>inicio_s</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>fin_s</t>
         </is>
@@ -1637,32 +1625,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>tren</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>ranura</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>t_esperado_s</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>t_medido_s</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>error_s</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>capturada</t>
         </is>
@@ -1783,27 +1771,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>evento</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>tiempo_s</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>amplitud_px</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>junto_a_hueco</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>junto_al_borde</t>
         </is>
@@ -1926,117 +1914,117 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>evento</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>grupo</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>tren</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>frame_pico</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>tiempo_s</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>amplitud_px</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>grosor_reposo_px</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>amplitud_relativa_pct</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>meseta_pico_frames</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>onset_s</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>ttp_frames</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>ttp_s</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>ttp_min_s</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>ttp_max_s</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>ttp_medible</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>rt50_frames</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>rt50_s</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>rt50_min_s</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>rt50_max_s</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>rt50_medible</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>offset_s</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>duracion_frames</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>duracion_s</t>
         </is>
@@ -2495,112 +2483,112 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>grupo</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>cinetica_min_frames</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>n_eventos_cinetica</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>amplitud_relativa_pct</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>amplitud_relativa_iqr_pct</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ttp_n_eventos</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>ttp_n_medibles</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>ttp_frames_mediana</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>ttp_reportable</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>ttp_s</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>ttp_iqr_s</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>ttp_cota_inf_s</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>ttp_cota_sup_s</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>rt50_n_eventos</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>rt50_n_medibles</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>rt50_frames_mediana</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>rt50_reportable</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>rt50_s</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>rt50_iqr_s</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>rt50_cota_inf_s</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>rt50_cota_sup_s</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>cinetica_motivo</t>
         </is>

</xml_diff>

<commit_message>
B6 aprobado (pico = primer fotograma >= 95% del maximo); basal; rotacion automatica para gel vertical; ventana: pulsos y comparar; resultados rehechos (paso 2)
</commit_message>
<xml_diff>
--- a/data/processed_data/Video_063_CTRL1_5V/contracciones_Video_063_CTRL1_5V.xlsx
+++ b/data/processed_data/Video_063_CTRL1_5V/contracciones_Video_063_CTRL1_5V.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="estab_Video_063_CTRL1_5V" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="resumen_Video_063_CTRL1_5V" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ritmo_Video_063_CTRL1_5V" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="trenes_Video_063_CTRL1_5V" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="grilla_Video_063_CTRL1_5V" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="eventos_Video_063_CTRL1_5V" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="cinetica_Video_063_CTRL1_5V" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="cin_grupos_Video_063_CTRL1_" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="estab_Video_063_CTRL1_5V" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="resumen_Video_063_CTRL1_5V" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ritmo_Video_063_CTRL1_5V" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="trenes_Video_063_CTRL1_5V" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="grilla_Video_063_CTRL1_5V" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="eventos_Video_063_CTRL1_5V" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="basal_Video_063_CTRL1_5V" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cinetica_Video_063_CTRL1_5V" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cin_grupos_Video_063_CTRL1_" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -778,7 +779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BL2"/>
+  <dimension ref="A1:CA2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -944,162 +945,237 @@
       </c>
       <c r="AG1" t="inlineStr">
         <is>
+          <t>amplitud_relativa_ic95_pct</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>amplitud_px</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
           <t>ttp_n_eventos</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>ttp_n_medibles</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>ttp_frames_mediana</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>ttp_reportable</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>ttp_s</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>ttp_iqr_s</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>ttp_ic95_s</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
         <is>
           <t>ttp_cota_inf_s</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>ttp_cota_sup_s</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>rt50_n_eventos</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>rt50_n_medibles</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>rt50_frames_mediana</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>rt50_reportable</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>rt50_s</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>rt50_iqr_s</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>rt50_ic95_s</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
         <is>
           <t>rt50_cota_inf_s</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>rt50_cota_sup_s</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>cinetica_motivo</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>fotogramas_sin_medida</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>fotogramas_sin_medida_pct</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>fotogramas_low_quality</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>eventos_junto_a_hueco</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>eventos_junto_al_borde</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>win_s_usado</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>win_s_automatico</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>duracion_evento_max_s</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>ventana_corta</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>conteo_por_ventana</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>conteo_estable_ventana</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>mesetas</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BN1" t="inlineStr">
         <is>
           <t>ruido_borde_sup_px</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
+      <c r="BO1" t="inlineStr">
         <is>
           <t>ruido_borde_inf_px</t>
         </is>
       </c>
-      <c r="BL1" t="inlineStr">
+      <c r="BP1" t="inlineStr">
         <is>
           <t>cociente_ruido_bordes</t>
+        </is>
+      </c>
+      <c r="BQ1" t="inlineStr">
+        <is>
+          <t>basal_fin_s</t>
+        </is>
+      </c>
+      <c r="BR1" t="inlineStr">
+        <is>
+          <t>basal_definicion</t>
+        </is>
+      </c>
+      <c r="BS1" t="inlineStr">
+        <is>
+          <t>basal_actividad_p95_px</t>
+        </is>
+      </c>
+      <c r="BT1" t="inlineStr">
+        <is>
+          <t>basal_actividad_p95_pct</t>
+        </is>
+      </c>
+      <c r="BU1" t="inlineStr">
+        <is>
+          <t>basal_contable</t>
+        </is>
+      </c>
+      <c r="BV1" t="inlineStr">
+        <is>
+          <t>basal_n_contracciones</t>
+        </is>
+      </c>
+      <c r="BW1" t="inlineStr">
+        <is>
+          <t>basal_instantes_s</t>
+        </is>
+      </c>
+      <c r="BX1" t="inlineStr">
+        <is>
+          <t>basal_junto_al_borde</t>
+        </is>
+      </c>
+      <c r="BY1" t="inlineStr">
+        <is>
+          <t>basal_amplitud_mediana_pct</t>
+        </is>
+      </c>
+      <c r="BZ1" t="inlineStr">
+        <is>
+          <t>basal_amplitud_mediana_px</t>
+        </is>
+      </c>
+      <c r="CA1" t="inlineStr">
+        <is>
+          <t>basal_resumen</t>
         </is>
       </c>
     </row>
@@ -1229,99 +1305,148 @@
           <t>0.5627-0.5819</t>
         </is>
       </c>
-      <c r="AG2" t="n">
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>0.523-0.5827</t>
+        </is>
+      </c>
+      <c r="AH2" t="n">
+        <v>1.591499999999996</v>
+      </c>
+      <c r="AI2" t="n">
         <v>5</v>
       </c>
-      <c r="AH2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI2" t="n">
+      <c r="AJ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK2" t="n">
         <v>2</v>
       </c>
-      <c r="AJ2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN2" t="n">
+      <c r="AL2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ2" t="n">
         <v>0.09999999999999964</v>
       </c>
-      <c r="AO2" t="n">
+      <c r="AR2" t="n">
         <v>5</v>
       </c>
-      <c r="AP2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ2" t="n">
+      <c r="AS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT2" t="n">
         <v>2</v>
       </c>
-      <c r="AR2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV2" t="n">
+      <c r="AU2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ2" t="n">
         <v>0.1000000000000014</v>
       </c>
-      <c r="AW2" t="inlineStr">
+      <c r="BA2" t="inlineStr">
         <is>
           <t>TTP: medible en 0 de 5 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota TTP &lt; 100 ms; RT50: medible en 0 de 5 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota RT50 &lt; 100 ms</t>
         </is>
       </c>
-      <c r="AX2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA2" t="n">
-        <v>0</v>
-      </c>
       <c r="BB2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG2" t="n">
         <v>2</v>
       </c>
-      <c r="BD2" t="b">
-        <v>1</v>
-      </c>
-      <c r="BE2" t="n">
+      <c r="BH2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BI2" t="n">
         <v>0.2333333333333201</v>
       </c>
-      <c r="BF2" t="b">
-        <v>0</v>
-      </c>
-      <c r="BG2" t="inlineStr">
+      <c r="BJ2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BK2" t="inlineStr">
         <is>
           <t>1.5 s: 6 | 2 s: 6 | 3 s: 6</t>
         </is>
       </c>
-      <c r="BH2" t="b">
-        <v>1</v>
-      </c>
-      <c r="BI2" t="inlineStr">
+      <c r="BL2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BM2" t="inlineStr">
         <is>
           <t>6 ev en k=9.415-13.785; 5 ev en k=15.163-24.421</t>
         </is>
       </c>
-      <c r="BJ2" t="n">
+      <c r="BN2" t="n">
         <v>0.03513762000002872</v>
       </c>
-      <c r="BK2" t="n">
+      <c r="BO2" t="n">
         <v>0.03217241999984601</v>
       </c>
-      <c r="BL2" t="n">
+      <c r="BP2" t="n">
         <v>1.092165898623632</v>
+      </c>
+      <c r="BQ2" t="n">
+        <v>10</v>
+      </c>
+      <c r="BR2" t="inlineStr">
+        <is>
+          <t>0-10 s</t>
+        </is>
+      </c>
+      <c r="BS2" t="n">
+        <v>0.05277999999998997</v>
+      </c>
+      <c r="BT2" t="n">
+        <v>0.01870207713549188</v>
+      </c>
+      <c r="BU2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BV2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW2" t="inlineStr">
+        <is>
+          <t>0.31</t>
+        </is>
+      </c>
+      <c r="BX2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY2" t="n">
+        <v>0.1284245301778257</v>
+      </c>
+      <c r="BZ2" t="n">
+        <v>0.3624500000000239</v>
+      </c>
+      <c r="CA2" t="inlineStr">
+        <is>
+          <t>1 contraccion(es) en 10.0 s; amplitud mediana 0.13 %; actividad basal 0.02 % del grosor</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1767,7 +1892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1796,6 +1921,16 @@
           <t>junto_al_borde</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>en_promedio</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>reportable</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1811,6 +1946,12 @@
         <v>0</v>
       </c>
       <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1830,6 +1971,12 @@
       <c r="E3" t="b">
         <v>0</v>
       </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1847,6 +1994,12 @@
       <c r="E4" t="b">
         <v>0</v>
       </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1864,6 +2017,12 @@
       <c r="E5" t="b">
         <v>0</v>
       </c>
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1881,6 +2040,12 @@
       <c r="E6" t="b">
         <v>0</v>
       </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1897,6 +2062,12 @@
       </c>
       <c r="E7" t="b">
         <v>0</v>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1910,562 +2081,151 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W7"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>evento</t>
+          <t>dato</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>grupo</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>tren</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>frame_pico</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>tiempo_s</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>amplitud_px</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>grosor_reposo_px</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>amplitud_relativa_pct</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>meseta_pico_frames</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>onset_s</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>ttp_frames</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>ttp_s</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>ttp_min_s</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>ttp_max_s</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>ttp_medible</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>rt50_frames</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>rt50_s</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>rt50_min_s</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>rt50_max_s</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>rt50_medible</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>offset_s</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>duracion_frames</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>duracion_s</t>
+          <t>valor</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>basal_fin_s</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>espontaneos</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="n">
-        <v>11</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.3083333333333333</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0.3624500000000239</v>
-      </c>
-      <c r="G2" t="n">
-        <v>282.2280132137918</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.1284245301778257</v>
-      </c>
-      <c r="I2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.2560361885790169</v>
-      </c>
-      <c r="K2" t="n">
-        <v>2</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0.0522971447543164</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.09999999999999998</v>
-      </c>
-      <c r="O2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0.04237293932553299</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0.09833333333333327</v>
-      </c>
-      <c r="T2" t="b">
-        <v>0</v>
-      </c>
-      <c r="U2" t="n">
-        <v>0.3705407346603723</v>
-      </c>
-      <c r="V2" t="n">
-        <v>4</v>
-      </c>
-      <c r="W2" t="n">
-        <v>0.1145045460813554</v>
+          <t>10.0</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>basal_definicion</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>estimulados</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" t="n">
-        <v>359</v>
-      </c>
-      <c r="E3" t="n">
-        <v>11.91166666666667</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1.644399999999962</v>
-      </c>
-      <c r="G3" t="n">
-        <v>282.2092391233975</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.582688222790941</v>
-      </c>
-      <c r="I3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" t="n">
-        <v>11.87549220051491</v>
-      </c>
-      <c r="K3" t="n">
-        <v>2</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0.03617446615175623</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.09999999999999964</v>
-      </c>
-      <c r="O3" t="b">
-        <v>0</v>
-      </c>
-      <c r="P3" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0.04801368061036193</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0.09666666666666934</v>
-      </c>
-      <c r="T3" t="b">
-        <v>0</v>
-      </c>
-      <c r="U3" t="n">
-        <v>12.01312337294851</v>
-      </c>
-      <c r="V3" t="n">
-        <v>6</v>
-      </c>
-      <c r="W3" t="n">
-        <v>0.1376311724335952</v>
+          <t>0-10 s</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>basal_actividad_p95_px</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>estimulados</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="n">
-        <v>659</v>
-      </c>
-      <c r="E4" t="n">
-        <v>21.91</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1.591499999999996</v>
-      </c>
-      <c r="G4" t="n">
-        <v>282.2652345330425</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.5638313916458219</v>
-      </c>
-      <c r="I4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="n">
-        <v>21.87821873127871</v>
-      </c>
-      <c r="K4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.03178126872129283</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0.06666666666666998</v>
-      </c>
-      <c r="O4" t="b">
-        <v>0</v>
-      </c>
-      <c r="P4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.05053973302491954</v>
-      </c>
-      <c r="R4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" t="n">
-        <v>0.1000000000000014</v>
-      </c>
-      <c r="T4" t="b">
-        <v>0</v>
-      </c>
-      <c r="U4" t="n">
-        <v>22.06191176470589</v>
-      </c>
-      <c r="V4" t="n">
-        <v>6</v>
-      </c>
-      <c r="W4" t="n">
-        <v>0.1836930334271862</v>
+          <t>0.05277999999998997</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>basal_actividad_p95_pct</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>estimulados</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" t="n">
-        <v>959</v>
-      </c>
-      <c r="E5" t="n">
-        <v>31.91</v>
-      </c>
-      <c r="F5" t="n">
-        <v>1.642200000000003</v>
-      </c>
-      <c r="G5" t="n">
-        <v>282.1992089136095</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.5819293421558578</v>
-      </c>
-      <c r="I5" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" t="n">
-        <v>31.86843231162197</v>
-      </c>
-      <c r="K5" t="n">
-        <v>2</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.04156768837803426</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.1000000000000085</v>
-      </c>
-      <c r="O5" t="b">
-        <v>0</v>
-      </c>
-      <c r="P5" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0.05105462412115358</v>
-      </c>
-      <c r="R5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" t="n">
-        <v>0.1000000000000014</v>
-      </c>
-      <c r="T5" t="b">
-        <v>0</v>
-      </c>
-      <c r="U5" t="n">
-        <v>32.01879704301076</v>
-      </c>
-      <c r="V5" t="n">
-        <v>6</v>
-      </c>
-      <c r="W5" t="n">
-        <v>0.1503647313887981</v>
+          <t>0.018702077135491883</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>basal_contable</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>estimulados</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" t="n">
-        <v>1259</v>
-      </c>
-      <c r="E6" t="n">
-        <v>41.90833333333334</v>
-      </c>
-      <c r="F6" t="n">
-        <v>1.476100000000031</v>
-      </c>
-      <c r="G6" t="n">
-        <v>282.2543039692085</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.5229681104033973</v>
-      </c>
-      <c r="I6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" t="n">
-        <v>41.87677143821742</v>
-      </c>
-      <c r="K6" t="n">
-        <v>1</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.03156189511591379</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0.06499999999999773</v>
-      </c>
-      <c r="O6" t="b">
-        <v>0</v>
-      </c>
-      <c r="P6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0.0517839004570817</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0.09833333333332916</v>
-      </c>
-      <c r="T6" t="b">
-        <v>0</v>
-      </c>
-      <c r="U6" t="n">
-        <v>42.02637431693989</v>
-      </c>
-      <c r="V6" t="n">
-        <v>5</v>
-      </c>
-      <c r="W6" t="n">
-        <v>0.1496028787224688</v>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>basal_n_contracciones</t>
+        </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>estimulados</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" t="n">
-        <v>1549</v>
-      </c>
-      <c r="E7" t="n">
-        <v>51.90833333333334</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1.588099999999997</v>
-      </c>
-      <c r="G7" t="n">
-        <v>282.2367268937121</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.5626836795758554</v>
-      </c>
-      <c r="I7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" t="n">
-        <v>51.86682667934094</v>
-      </c>
-      <c r="K7" t="n">
-        <v>2</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0.04150665399239983</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0.1000000000000014</v>
-      </c>
-      <c r="O7" t="b">
-        <v>0</v>
-      </c>
-      <c r="P7" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0.05077394072985442</v>
-      </c>
-      <c r="R7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0.1000000000000014</v>
-      </c>
-      <c r="T7" t="b">
-        <v>0</v>
-      </c>
-      <c r="U7" t="n">
-        <v>52.03418753365644</v>
-      </c>
-      <c r="V7" t="n">
-        <v>6</v>
-      </c>
-      <c r="W7" t="n">
-        <v>0.1673608543155041</v>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>basal_instantes_s</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0.31</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>basal_junto_al_borde</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>basal_amplitud_mediana_pct</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0.1284245301778257</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>basal_amplitud_mediana_px</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0.3624500000000239</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>basal_resumen</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1 contraccion(es) en 10.0 s; amplitud mediana 0.13 %; actividad basal 0.02 % del grosor</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2479,15 +2239,653 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:Z7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>evento</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>grupo</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>tren</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>frame_pico</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>tiempo_s</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>amplitud_px</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>grosor_reposo_px</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>amplitud_relativa_pct</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>meseta_pico_frames</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>frame_llega_max</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>tiempo_llega_max_s</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>pico_dudoso_por_ruido</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>onset_s</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>ttp_frames</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>ttp_s</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>ttp_min_s</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>ttp_max_s</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>ttp_medible</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>rt50_frames</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>rt50_s</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>rt50_min_s</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>rt50_max_s</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>rt50_medible</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>offset_s</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>duracion_frames</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>duracion_s</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>espontaneos</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.3083333333333333</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.3624500000000239</v>
+      </c>
+      <c r="G2" t="n">
+        <v>282.2280132137918</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.1284245301778257</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>11</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.3083333333333333</v>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.2560361885790169</v>
+      </c>
+      <c r="N2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.0522971447543164</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.09999999999999998</v>
+      </c>
+      <c r="R2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>2</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.04237293932553299</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.09833333333333327</v>
+      </c>
+      <c r="W2" t="b">
+        <v>0</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0.3705407346603723</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0.1145045460813554</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>estimulados</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>359</v>
+      </c>
+      <c r="E3" t="n">
+        <v>11.91166666666667</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.644399999999962</v>
+      </c>
+      <c r="G3" t="n">
+        <v>282.2092391233975</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.582688222790941</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>359</v>
+      </c>
+      <c r="K3" t="n">
+        <v>11.91166666666667</v>
+      </c>
+      <c r="L3" t="b">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>11.87549220051491</v>
+      </c>
+      <c r="N3" t="n">
+        <v>2</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.03617446615175623</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.09999999999999964</v>
+      </c>
+      <c r="R3" t="b">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
+        <v>2</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.04801368061036193</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.09666666666666934</v>
+      </c>
+      <c r="W3" t="b">
+        <v>0</v>
+      </c>
+      <c r="X3" t="n">
+        <v>12.01312337294851</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>0.1376311724335952</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>estimulados</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>659</v>
+      </c>
+      <c r="E4" t="n">
+        <v>21.91</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1.591499999999996</v>
+      </c>
+      <c r="G4" t="n">
+        <v>282.2652345330425</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.5638313916458219</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="n">
+        <v>659</v>
+      </c>
+      <c r="K4" t="n">
+        <v>21.91</v>
+      </c>
+      <c r="L4" t="b">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>21.87821873127871</v>
+      </c>
+      <c r="N4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.03178126872129283</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.06666666666666998</v>
+      </c>
+      <c r="R4" t="b">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.05053973302491954</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.1000000000000014</v>
+      </c>
+      <c r="W4" t="b">
+        <v>0</v>
+      </c>
+      <c r="X4" t="n">
+        <v>22.06191176470589</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>0.1836930334271862</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>estimulados</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>959</v>
+      </c>
+      <c r="E5" t="n">
+        <v>31.91</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1.642200000000003</v>
+      </c>
+      <c r="G5" t="n">
+        <v>282.1992089136095</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.5819293421558578</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="n">
+        <v>959</v>
+      </c>
+      <c r="K5" t="n">
+        <v>31.91</v>
+      </c>
+      <c r="L5" t="b">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>31.86843231162197</v>
+      </c>
+      <c r="N5" t="n">
+        <v>2</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.04156768837803426</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.1000000000000085</v>
+      </c>
+      <c r="R5" t="b">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
+        <v>2</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.05105462412115358</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.1000000000000014</v>
+      </c>
+      <c r="W5" t="b">
+        <v>0</v>
+      </c>
+      <c r="X5" t="n">
+        <v>32.01879704301076</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0.1503647313887981</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>estimulados</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1259</v>
+      </c>
+      <c r="E6" t="n">
+        <v>41.90833333333334</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.476100000000031</v>
+      </c>
+      <c r="G6" t="n">
+        <v>282.2543039692085</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.5229681104033973</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1259</v>
+      </c>
+      <c r="K6" t="n">
+        <v>41.90833333333334</v>
+      </c>
+      <c r="L6" t="b">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>41.87677143821742</v>
+      </c>
+      <c r="N6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.03156189511591379</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.06499999999999773</v>
+      </c>
+      <c r="R6" t="b">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
+        <v>2</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.0517839004570817</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.09833333333332916</v>
+      </c>
+      <c r="W6" t="b">
+        <v>0</v>
+      </c>
+      <c r="X6" t="n">
+        <v>42.02637431693989</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0.1496028787224688</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>estimulados</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1549</v>
+      </c>
+      <c r="E7" t="n">
+        <v>51.90833333333334</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.588099999999997</v>
+      </c>
+      <c r="G7" t="n">
+        <v>282.2367268937121</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.5626836795758554</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1549</v>
+      </c>
+      <c r="K7" t="n">
+        <v>51.90833333333334</v>
+      </c>
+      <c r="L7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>51.86682667934094</v>
+      </c>
+      <c r="N7" t="n">
+        <v>2</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.04150665399239983</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0.1000000000000014</v>
+      </c>
+      <c r="R7" t="b">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
+        <v>2</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0.05077394072985442</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0.1000000000000014</v>
+      </c>
+      <c r="W7" t="b">
+        <v>0</v>
+      </c>
+      <c r="X7" t="n">
+        <v>52.03418753365644</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>0.1673608543155041</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Z4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>grupo</t>
+        </is>
+      </c>
       <c r="B1" t="inlineStr">
         <is>
           <t>cinetica_min_frames</t>
@@ -2510,85 +2908,105 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>amplitud_relativa_ic95_pct</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>amplitud_px</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>ttp_n_eventos</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>ttp_n_medibles</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>ttp_frames_mediana</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>ttp_reportable</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>ttp_s</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>ttp_iqr_s</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>ttp_ic95_s</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
         <is>
           <t>ttp_cota_inf_s</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>ttp_cota_sup_s</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>rt50_n_eventos</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>rt50_n_medibles</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>rt50_frames_mediana</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>rt50_reportable</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>rt50_s</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>rt50_iqr_s</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>rt50_ic95_s</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
         <is>
           <t>rt50_cota_inf_s</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>rt50_cota_sup_s</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>cinetica_motivo</t>
         </is>
@@ -2614,47 +3032,57 @@
           <t>0.5329-0.5774</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.3257-0.5823</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>1.589799999999997</v>
+      </c>
+      <c r="H2" t="n">
         <v>6</v>
       </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
         <v>2</v>
       </c>
-      <c r="I2" t="b">
-        <v>0</v>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
+      <c r="K2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
         <v>0.09999999999999981</v>
       </c>
-      <c r="N2" t="n">
+      <c r="Q2" t="n">
         <v>6</v>
       </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
         <v>2</v>
       </c>
-      <c r="Q2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U2" t="n">
+      <c r="T2" t="b">
+        <v>0</v>
+      </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="n">
         <v>0.09916666666666735</v>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>TTP: medible en 0 de 6 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota TTP &lt; 100 ms; RT50: medible en 0 de 6 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota RT50 &lt; 99 ms</t>
         </is>
@@ -2680,47 +3108,57 @@
           <t>0.5627-0.5819</t>
         </is>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.523-0.5827</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1.591499999999996</v>
+      </c>
+      <c r="H3" t="n">
         <v>5</v>
       </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
         <v>2</v>
       </c>
-      <c r="I3" t="b">
-        <v>0</v>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="n">
+      <c r="K3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
         <v>0.09999999999999964</v>
       </c>
-      <c r="N3" t="n">
+      <c r="Q3" t="n">
         <v>5</v>
       </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="n">
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
         <v>2</v>
       </c>
-      <c r="Q3" t="b">
-        <v>0</v>
-      </c>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U3" t="n">
+      <c r="T3" t="b">
+        <v>0</v>
+      </c>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="n">
         <v>0.1000000000000014</v>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="Z3" t="inlineStr">
         <is>
           <t>TTP: medible en 0 de 5 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota TTP &lt; 100 ms; RT50: medible en 0 de 5 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota RT50 &lt; 100 ms</t>
         </is>
@@ -2742,47 +3180,53 @@
         <v>0.1284245301778257</v>
       </c>
       <c r="E4" t="inlineStr"/>
-      <c r="F4" t="n">
-        <v>1</v>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>0.3624500000000239</v>
       </c>
       <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
         <v>2</v>
       </c>
-      <c r="I4" t="b">
-        <v>0</v>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" t="n">
+      <c r="K4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
         <v>0.09999999999999998</v>
       </c>
-      <c r="N4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
         <v>2</v>
       </c>
-      <c r="Q4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U4" t="n">
+      <c r="T4" t="b">
+        <v>0</v>
+      </c>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="n">
         <v>0.09833333333333327</v>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>TTP: medible en 0 de 1 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota TTP &lt; 100 ms; RT50: medible en 0 de 1 eventos (&lt; la mitad con &gt;= 5 fotogramas); solo cota RT50 &lt; 98 ms</t>
         </is>

</xml_diff>